<commit_message>
Add comments for calculation
</commit_message>
<xml_diff>
--- a/docs/assets/images/User_description/Consumption_and_autonomy.xlsx
+++ b/docs/assets/images/User_description/Consumption_and_autonomy.xlsx
@@ -67,6 +67,50 @@
         </r>
       </text>
     </comment>
+    <comment ref="E34" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">Current = leakage current of component + Equivalent dissipated current
+Equivalent dissipated current = Power dissipated by regulator / Input voltage 
+Power dissipated by regulator = ΔU x I consumed by emitter &amp; receiver
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G39" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Power consumed = Leakage current x Input voltage + Power provided / (1 - Efficiency)
+This is the max power provided : We consider the RFID reader inthe mode where its consumption is the highest.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I39" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Energy consumed = Leakage current x Input voltage x Duration + Energy provided / (1 - Efficiency)
+The power consumption cannot be directly used for this calculation, as the power board does not provide this power all the time (it's only the max)</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -235,7 +279,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -317,6 +361,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -605,6 +655,57 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -629,62 +730,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -748,6 +798,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -841,6 +892,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -1958,22 +2010,22 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:15" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="44"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="M2" s="60"/>
+      <c r="N2" s="60"/>
+      <c r="O2" s="61"/>
     </row>
     <row r="4" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="8" t="s">
@@ -1996,24 +2048,24 @@
       <c r="O4" s="1"/>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="38"/>
+      <c r="C6" s="55"/>
       <c r="D6" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="63" t="s">
+      <c r="E6" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="63"/>
+      <c r="F6" s="38"/>
       <c r="G6" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="37" t="s">
+      <c r="J6" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="K6" s="38"/>
+      <c r="K6" s="55"/>
       <c r="L6" s="30" t="s">
         <v>46</v>
       </c>
@@ -2025,17 +2077,17 @@
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="51"/>
+      <c r="C7" s="44"/>
       <c r="D7" s="17">
         <v>5</v>
       </c>
-      <c r="E7" s="61">
+      <c r="E7" s="37">
         <v>13</v>
       </c>
-      <c r="F7" s="61"/>
+      <c r="F7" s="37"/>
       <c r="G7" s="10">
         <f t="shared" ref="G7:G14" si="0">E7*D7</f>
         <v>65</v>
@@ -2055,17 +2107,17 @@
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="50" t="s">
+      <c r="B8" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="51"/>
+      <c r="C8" s="44"/>
       <c r="D8" s="17">
         <v>5</v>
       </c>
-      <c r="E8" s="61">
+      <c r="E8" s="37">
         <v>16</v>
       </c>
-      <c r="F8" s="61"/>
+      <c r="F8" s="37"/>
       <c r="G8" s="10">
         <f t="shared" si="0"/>
         <v>80</v>
@@ -2085,102 +2137,102 @@
       </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="53"/>
+      <c r="C9" s="48"/>
       <c r="D9" s="17">
         <v>5</v>
       </c>
-      <c r="E9" s="61">
+      <c r="E9" s="37">
         <v>77.5</v>
       </c>
-      <c r="F9" s="61"/>
+      <c r="F9" s="37"/>
       <c r="G9" s="10">
         <f t="shared" si="0"/>
         <v>387.5</v>
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="50" t="s">
+      <c r="B10" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="51"/>
+      <c r="C10" s="44"/>
       <c r="D10" s="17">
         <v>5</v>
       </c>
-      <c r="E10" s="61">
+      <c r="E10" s="37">
         <v>46.5</v>
       </c>
-      <c r="F10" s="61"/>
+      <c r="F10" s="37"/>
       <c r="G10" s="10">
         <f t="shared" si="0"/>
         <v>232.5</v>
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="52" t="s">
+      <c r="B11" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="53"/>
+      <c r="C11" s="48"/>
       <c r="D11" s="17">
         <v>3.3</v>
       </c>
-      <c r="E11" s="61">
+      <c r="E11" s="37">
         <v>4.8</v>
       </c>
-      <c r="F11" s="61"/>
+      <c r="F11" s="37"/>
       <c r="G11" s="10">
         <f t="shared" si="0"/>
         <v>15.839999999999998</v>
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="52" t="s">
+      <c r="B12" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="53"/>
+      <c r="C12" s="48"/>
       <c r="D12" s="17">
         <v>3.3</v>
       </c>
-      <c r="E12" s="60">
+      <c r="E12" s="39">
         <v>0.4</v>
       </c>
-      <c r="F12" s="60"/>
+      <c r="F12" s="39"/>
       <c r="G12" s="10">
         <f t="shared" si="0"/>
         <v>1.32</v>
       </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="52" t="s">
+      <c r="B13" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="53"/>
+      <c r="C13" s="48"/>
       <c r="D13" s="17">
         <v>5</v>
       </c>
-      <c r="E13" s="60">
+      <c r="E13" s="39">
         <v>5.5</v>
       </c>
-      <c r="F13" s="60"/>
+      <c r="F13" s="39"/>
       <c r="G13" s="10">
         <f t="shared" si="0"/>
         <v>27.5</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="50" t="s">
+      <c r="B14" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="51"/>
+      <c r="C14" s="44"/>
       <c r="D14" s="17">
         <v>3.6</v>
       </c>
-      <c r="E14" s="60">
+      <c r="E14" s="39">
         <v>5</v>
       </c>
-      <c r="F14" s="60"/>
+      <c r="F14" s="39"/>
       <c r="G14" s="10">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2213,25 +2265,25 @@
       <c r="O17" s="1"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="40"/>
-      <c r="D19" s="41"/>
-      <c r="F19" s="39" t="s">
+      <c r="C19" s="57"/>
+      <c r="D19" s="58"/>
+      <c r="F19" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="G19" s="40"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="41"/>
-      <c r="K19" s="39" t="s">
+      <c r="G19" s="57"/>
+      <c r="H19" s="57"/>
+      <c r="I19" s="58"/>
+      <c r="K19" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="L19" s="40" t="s">
+      <c r="L19" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="M19" s="40"/>
-      <c r="N19" s="41"/>
+      <c r="M19" s="57"/>
+      <c r="N19" s="58"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B20" s="11"/>
@@ -2381,17 +2433,17 @@
       <c r="O29" s="1"/>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B31" s="47" t="s">
+      <c r="B31" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="C31" s="48"/>
+      <c r="C31" s="63"/>
       <c r="D31" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="62" t="s">
+      <c r="E31" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="F31" s="62"/>
+      <c r="F31" s="45"/>
       <c r="G31" s="25" t="s">
         <v>27</v>
       </c>
@@ -2408,19 +2460,19 @@
       </c>
     </row>
     <row r="32" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B32" s="45" t="s">
+      <c r="B32" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="C32" s="46"/>
+      <c r="C32" s="41"/>
       <c r="D32" s="21">
         <f>D11</f>
         <v>3.3</v>
       </c>
-      <c r="E32" s="49">
+      <c r="E32" s="42">
         <f>2*IF(OR(D21,D22),E11,0)</f>
         <v>9.6</v>
       </c>
-      <c r="F32" s="49"/>
+      <c r="F32" s="42"/>
       <c r="G32" s="21">
         <f>D32*E32</f>
         <v>31.679999999999996</v>
@@ -2429,31 +2481,31 @@
         <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)</f>
         <v>24</v>
       </c>
-      <c r="I32" s="49">
+      <c r="I32" s="42">
         <f>G32*H32</f>
         <v>760.31999999999994</v>
       </c>
-      <c r="J32" s="49"/>
-      <c r="K32" s="49"/>
+      <c r="J32" s="42"/>
+      <c r="K32" s="42"/>
       <c r="L32" s="27">
         <f t="shared" ref="L32:L39" si="1">I32/1000/$D$41</f>
         <v>0.12999515572906273</v>
       </c>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B33" s="45" t="s">
+      <c r="B33" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="46"/>
+      <c r="C33" s="41"/>
       <c r="D33" s="21">
         <f>D12</f>
         <v>3.3</v>
       </c>
-      <c r="E33" s="49">
+      <c r="E33" s="42">
         <f>2*IF(OR(D21,D22,D23),E12,0)</f>
         <v>0.8</v>
       </c>
-      <c r="F33" s="49"/>
+      <c r="F33" s="42"/>
       <c r="G33" s="21">
         <f t="shared" ref="G33:G38" si="2">D33*E33</f>
         <v>2.64</v>
@@ -2462,31 +2514,31 @@
         <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)</f>
         <v>24</v>
       </c>
-      <c r="I33" s="49">
+      <c r="I33" s="42">
         <f t="shared" ref="I33:I38" si="3">G33*H33</f>
         <v>63.36</v>
       </c>
-      <c r="J33" s="49"/>
-      <c r="K33" s="49"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42"/>
       <c r="L33" s="27">
         <f t="shared" si="1"/>
         <v>1.0832929644088564E-2</v>
       </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B34" s="45" t="s">
+      <c r="B34" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="46"/>
+      <c r="C34" s="41"/>
       <c r="D34" s="21">
         <f>D13</f>
         <v>5</v>
       </c>
-      <c r="E34" s="58">
+      <c r="E34" s="53">
         <f>IF(OR(D21,D22,D23),E13+(E32+E33)*(D34-D33)/D34,0)</f>
         <v>9.0360000000000014</v>
       </c>
-      <c r="F34" s="58"/>
+      <c r="F34" s="53"/>
       <c r="G34" s="21">
         <f t="shared" si="2"/>
         <v>45.180000000000007</v>
@@ -2495,31 +2547,31 @@
         <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)</f>
         <v>24</v>
       </c>
-      <c r="I34" s="49">
+      <c r="I34" s="42">
         <f t="shared" si="3"/>
         <v>1084.3200000000002</v>
       </c>
-      <c r="J34" s="49"/>
-      <c r="K34" s="49"/>
+      <c r="J34" s="42"/>
+      <c r="K34" s="42"/>
       <c r="L34" s="27">
         <f t="shared" si="1"/>
         <v>0.18539081868178839</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C35" s="46"/>
+      <c r="C35" s="41"/>
       <c r="D35" s="21">
         <f t="shared" ref="D35:E38" si="4">D7</f>
         <v>5</v>
       </c>
-      <c r="E35" s="49">
+      <c r="E35" s="42">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="F35" s="49"/>
+      <c r="F35" s="42"/>
       <c r="G35" s="21">
         <f t="shared" si="2"/>
         <v>65</v>
@@ -2527,31 +2579,31 @@
       <c r="H35" s="21">
         <v>24</v>
       </c>
-      <c r="I35" s="49">
+      <c r="I35" s="42">
         <f t="shared" si="3"/>
         <v>1560</v>
       </c>
-      <c r="J35" s="49"/>
-      <c r="K35" s="49"/>
+      <c r="J35" s="42"/>
+      <c r="K35" s="42"/>
       <c r="L35" s="27">
         <f t="shared" si="1"/>
         <v>0.26671985866127146</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B36" s="45" t="s">
+      <c r="B36" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="C36" s="46"/>
+      <c r="C36" s="41"/>
       <c r="D36" s="21">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E36" s="49">
+      <c r="E36" s="42">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="F36" s="49"/>
+      <c r="F36" s="42"/>
       <c r="G36" s="21">
         <f t="shared" si="2"/>
         <v>80</v>
@@ -2560,31 +2612,31 @@
         <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)-H37-H38</f>
         <v>22.333333333333336</v>
       </c>
-      <c r="I36" s="49">
+      <c r="I36" s="42">
         <f t="shared" si="3"/>
         <v>1786.666666666667</v>
       </c>
-      <c r="J36" s="49"/>
-      <c r="K36" s="49"/>
+      <c r="J36" s="42"/>
+      <c r="K36" s="42"/>
       <c r="L36" s="27">
         <f t="shared" si="1"/>
         <v>0.30547402615906311</v>
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B37" s="45" t="s">
+      <c r="B37" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="C37" s="46"/>
+      <c r="C37" s="41"/>
       <c r="D37" s="21">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E37" s="49">
+      <c r="E37" s="42">
         <f t="shared" si="4"/>
         <v>77.5</v>
       </c>
-      <c r="F37" s="49"/>
+      <c r="F37" s="42"/>
       <c r="G37" s="21">
         <f t="shared" si="2"/>
         <v>387.5</v>
@@ -2593,31 +2645,31 @@
         <f>IF(NOT(OR(D21,D22)),IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)-H38,IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)*M21*(M22-M23)/3600)</f>
         <v>1.3333333333333333</v>
       </c>
-      <c r="I37" s="49">
+      <c r="I37" s="42">
         <f t="shared" si="3"/>
         <v>516.66666666666663</v>
       </c>
-      <c r="J37" s="49"/>
-      <c r="K37" s="49"/>
+      <c r="J37" s="42"/>
+      <c r="K37" s="42"/>
       <c r="L37" s="27">
         <f t="shared" si="1"/>
         <v>8.8336705325848433E-2</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B38" s="45" t="s">
+      <c r="B38" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="C38" s="46"/>
+      <c r="C38" s="41"/>
       <c r="D38" s="21">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E38" s="49">
+      <c r="E38" s="42">
         <f t="shared" si="4"/>
         <v>46.5</v>
       </c>
-      <c r="F38" s="49"/>
+      <c r="F38" s="42"/>
       <c r="G38" s="21">
         <f t="shared" si="2"/>
         <v>232.5</v>
@@ -2626,64 +2678,64 @@
         <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)*M21*M23/3600</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="I38" s="49">
+      <c r="I38" s="42">
         <f t="shared" si="3"/>
         <v>77.5</v>
       </c>
-      <c r="J38" s="49"/>
-      <c r="K38" s="49"/>
+      <c r="J38" s="42"/>
+      <c r="K38" s="42"/>
       <c r="L38" s="27">
         <f t="shared" si="1"/>
         <v>1.3250505798877267E-2</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B39" s="45" t="s">
+      <c r="B39" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="C39" s="46"/>
+      <c r="C39" s="41"/>
       <c r="D39" s="21">
         <f>H22</f>
         <v>12</v>
       </c>
-      <c r="E39" s="49">
+      <c r="E39" s="42">
         <f>IF(D39=12,0,E14)</f>
         <v>0</v>
       </c>
-      <c r="F39" s="49"/>
+      <c r="F39" s="42"/>
       <c r="G39" s="32">
-        <f>D39*E39+(1-IF(D39=12,M8,M7))*SUM(G32:G38)</f>
-        <v>177.34499999999997</v>
+        <f>D39*E39+(1-IF(D39=12,M8,M7))*(SUM(G32:G35)+MAX(G36:G38))</f>
+        <v>111.71999999999998</v>
       </c>
       <c r="H39" s="21">
         <v>24</v>
       </c>
-      <c r="I39" s="59">
+      <c r="I39" s="46">
         <f>D39*E39*H39+(1-IF(D39=12,M8,M7))*SUM(I32:K38)</f>
         <v>1228.2549999999999</v>
       </c>
-      <c r="J39" s="59"/>
-      <c r="K39" s="59"/>
+      <c r="J39" s="46"/>
+      <c r="K39" s="46"/>
       <c r="L39" s="27">
         <f t="shared" si="1"/>
         <v>0.20999999999999994</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B41" s="56" t="s">
+      <c r="B41" s="51" t="s">
         <v>30</v>
       </c>
-      <c r="C41" s="57"/>
+      <c r="C41" s="52"/>
       <c r="D41" s="3">
         <f>SUM(I32:I38)/1000</f>
         <v>5.8488333333333342</v>
       </c>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B42" s="54" t="s">
+      <c r="B42" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="C42" s="55"/>
+      <c r="C42" s="50"/>
       <c r="D42" s="2" t="str">
         <f>INT(H23/D41) &amp; "d " &amp; INT(24*MOD(H23,D41)/D41) &amp; "h " &amp; INT(MOD(24*60*MOD(H23,D41)/D41,60)) &amp; "m " &amp; INT(MOD(24*60*60*MOD(H23,D41)/D41,60)) &amp; "s"</f>
         <v>11d 1h 53m 57s</v>
@@ -2691,41 +2743,6 @@
     </row>
   </sheetData>
   <mergeCells count="51">
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E34:F34"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="F19:I19"/>
     <mergeCell ref="K19:N19"/>
@@ -2742,6 +2759,41 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="E10:F10"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D21:D24">

</xml_diff>

<commit_message>
Consumption correction for power boards
</commit_message>
<xml_diff>
--- a/docs/assets/images/User_description/Consumption_and_autonomy.xlsx
+++ b/docs/assets/images/User_description/Consumption_and_autonomy.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\btenaud\Documents\02 - Projet Antenne-Terrier\02 - Git\rfid_m0.wiki\docs\assets\images\User_description\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\btenaud\Documents\02 - Projet Antenne-Terrier\05 - Documents\2023.04.26 - Estimation conso &amp; autonomie\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -67,7 +67,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E34" authorId="0" shapeId="0">
+    <comment ref="E33" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -83,7 +83,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G39" authorId="0" shapeId="0">
+    <comment ref="G38" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -97,7 +97,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I39" authorId="0" shapeId="0">
+    <comment ref="I38" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -116,7 +116,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="48">
   <si>
     <t>Component</t>
   </si>
@@ -655,86 +655,86 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -913,7 +913,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Feuil1!$B$32:$C$39</c:f>
+              <c:f>Feuil1!$B$31:$C$38</c:f>
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
@@ -945,7 +945,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$L$32:$L$39</c:f>
+              <c:f>Feuil1!$L$31:$L$38</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="8"/>
@@ -1697,13 +1697,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>390525</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>104774</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>266700</xdr:colOff>
-      <xdr:row>60</xdr:row>
+      <xdr:row>59</xdr:row>
       <xdr:rowOff>152399</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1989,7 +1989,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:O42"/>
+  <dimension ref="B1:O41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2010,22 +2010,22 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:15" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="M2" s="60"/>
-      <c r="N2" s="60"/>
-      <c r="O2" s="61"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="44"/>
     </row>
     <row r="4" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="8" t="s">
@@ -2048,24 +2048,24 @@
       <c r="O4" s="1"/>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="55"/>
+      <c r="C6" s="38"/>
       <c r="D6" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="38" t="s">
+      <c r="E6" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="38"/>
+      <c r="F6" s="63"/>
       <c r="G6" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="54" t="s">
+      <c r="J6" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="K6" s="55"/>
+      <c r="K6" s="38"/>
       <c r="L6" s="30" t="s">
         <v>46</v>
       </c>
@@ -2077,19 +2077,19 @@
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="44"/>
+      <c r="C7" s="51"/>
       <c r="D7" s="17">
         <v>5</v>
       </c>
-      <c r="E7" s="37">
+      <c r="E7" s="61">
         <v>13</v>
       </c>
-      <c r="F7" s="37"/>
+      <c r="F7" s="61"/>
       <c r="G7" s="10">
-        <f t="shared" ref="G7:G14" si="0">E7*D7</f>
+        <f t="shared" ref="G7:G13" si="0">E7*D7</f>
         <v>65</v>
       </c>
       <c r="J7" s="9" t="s">
@@ -2107,17 +2107,17 @@
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="43" t="s">
+      <c r="B8" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="44"/>
+      <c r="C8" s="51"/>
       <c r="D8" s="17">
         <v>5</v>
       </c>
-      <c r="E8" s="37">
+      <c r="E8" s="61">
         <v>16</v>
       </c>
-      <c r="F8" s="37"/>
+      <c r="F8" s="61"/>
       <c r="G8" s="10">
         <f t="shared" si="0"/>
         <v>80</v>
@@ -2137,621 +2137,636 @@
       </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="47" t="s">
+      <c r="B9" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="48"/>
+      <c r="C9" s="53"/>
       <c r="D9" s="17">
         <v>5</v>
       </c>
-      <c r="E9" s="37">
+      <c r="E9" s="61">
         <v>77.5</v>
       </c>
-      <c r="F9" s="37"/>
+      <c r="F9" s="61"/>
       <c r="G9" s="10">
         <f t="shared" si="0"/>
         <v>387.5</v>
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="43" t="s">
+      <c r="B10" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="44"/>
+      <c r="C10" s="51"/>
       <c r="D10" s="17">
         <v>5</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="61">
         <v>46.5</v>
       </c>
-      <c r="F10" s="37"/>
+      <c r="F10" s="61"/>
       <c r="G10" s="10">
         <f t="shared" si="0"/>
         <v>232.5</v>
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="47" t="s">
+      <c r="B11" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="48"/>
+      <c r="C11" s="53"/>
       <c r="D11" s="17">
         <v>3.3</v>
       </c>
-      <c r="E11" s="37">
+      <c r="E11" s="61">
         <v>4.8</v>
       </c>
-      <c r="F11" s="37"/>
+      <c r="F11" s="61"/>
       <c r="G11" s="10">
         <f t="shared" si="0"/>
         <v>15.839999999999998</v>
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="47" t="s">
+      <c r="B12" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="48"/>
+      <c r="C12" s="53"/>
       <c r="D12" s="17">
         <v>3.3</v>
       </c>
-      <c r="E12" s="39">
+      <c r="E12" s="60">
         <v>0.4</v>
       </c>
-      <c r="F12" s="39"/>
+      <c r="F12" s="60"/>
       <c r="G12" s="10">
         <f t="shared" si="0"/>
         <v>1.32</v>
       </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="47" t="s">
+      <c r="B13" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="48"/>
+      <c r="C13" s="53"/>
       <c r="D13" s="17">
         <v>5</v>
       </c>
-      <c r="E13" s="39">
+      <c r="E13" s="60">
         <v>5.5</v>
       </c>
-      <c r="F13" s="39"/>
+      <c r="F13" s="60"/>
       <c r="G13" s="10">
         <f t="shared" si="0"/>
         <v>27.5</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="17">
-        <v>3.6</v>
-      </c>
-      <c r="E14" s="39">
-        <v>5</v>
-      </c>
-      <c r="F14" s="39"/>
-      <c r="G14" s="10">
-        <f t="shared" si="0"/>
-        <v>18</v>
+      <c r="B14" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="4"/>
-    </row>
-    <row r="17" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B17" s="8" t="s">
+      <c r="B15" s="4"/>
+    </row>
+    <row r="16" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B16" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="40"/>
+      <c r="D18" s="41"/>
+      <c r="F18" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="41"/>
+      <c r="K18" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="L18" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="M18" s="40"/>
+      <c r="N18" s="41"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="56" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="57"/>
-      <c r="D19" s="58"/>
-      <c r="F19" s="56" t="s">
-        <v>32</v>
-      </c>
-      <c r="G19" s="57"/>
-      <c r="H19" s="57"/>
-      <c r="I19" s="58"/>
-      <c r="K19" s="56" t="s">
-        <v>33</v>
-      </c>
-      <c r="L19" s="57" t="s">
-        <v>10</v>
-      </c>
-      <c r="M19" s="57"/>
-      <c r="N19" s="58"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="15"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="20"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="20"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B20" s="11"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="15"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="13" t="b">
+        <v>1</v>
+      </c>
       <c r="F20" s="12"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
+      <c r="G20" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" s="7">
+        <v>5.4</v>
+      </c>
       <c r="I20" s="20"/>
       <c r="K20" s="12"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
+      <c r="L20" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="M20" s="7">
+        <v>50</v>
+      </c>
       <c r="N20" s="20"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B21" s="12"/>
       <c r="C21" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D21" s="13" t="b">
         <v>1</v>
       </c>
       <c r="F21" s="12"/>
       <c r="G21" s="5" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H21" s="7">
-        <v>5.4</v>
+        <v>12</v>
       </c>
       <c r="I21" s="20"/>
       <c r="K21" s="12"/>
       <c r="L21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="M21" s="7">
         <v>5</v>
-      </c>
-      <c r="M21" s="7">
-        <v>50</v>
       </c>
       <c r="N21" s="20"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B22" s="12"/>
       <c r="C22" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D22" s="13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" s="12"/>
       <c r="G22" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H22" s="7">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="H22" s="19">
+        <f>H20*H21</f>
+        <v>64.800000000000011</v>
       </c>
       <c r="I22" s="20"/>
       <c r="K22" s="12"/>
       <c r="L22" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="M22" s="7">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="M22" s="36">
+        <v>1</v>
       </c>
       <c r="N22" s="20"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B23" s="12"/>
       <c r="C23" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D23" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="F23" s="12"/>
-      <c r="G23" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="H23" s="19">
-        <f>H21*H22</f>
-        <v>64.800000000000011</v>
-      </c>
-      <c r="I23" s="20"/>
-      <c r="K23" s="12"/>
-      <c r="L23" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="M23" s="36">
-        <v>1</v>
-      </c>
-      <c r="N23" s="20"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="16"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="16"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B24" s="12"/>
       <c r="C24" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D24" s="13" t="b">
-        <v>0</v>
-      </c>
-      <c r="F24" s="14"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="16"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="16"/>
+        <v>19</v>
+      </c>
+      <c r="D24" s="13">
+        <v>8</v>
+      </c>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B25" s="12"/>
       <c r="C25" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="12"/>
-      <c r="C26" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D26" s="13">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B27" s="14"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="16"/>
-    </row>
-    <row r="29" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B29" s="8" t="s">
+      <c r="B26" s="14"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="16"/>
+    </row>
+    <row r="28" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B28" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C29" s="18"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B30" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="C30" s="48"/>
+      <c r="D30" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" s="62" t="s">
+        <v>34</v>
+      </c>
+      <c r="F30" s="62"/>
+      <c r="G30" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="H30" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="I30" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="J30" s="24"/>
+      <c r="K30" s="24"/>
+      <c r="L30" s="26" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B31" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="63"/>
-      <c r="D31" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="E31" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="F31" s="45"/>
-      <c r="G31" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="H31" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="I31" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="J31" s="24"/>
-      <c r="K31" s="24"/>
-      <c r="L31" s="26" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B32" s="40" t="s">
+      <c r="B31" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="C32" s="41"/>
-      <c r="D32" s="21">
+      <c r="C31" s="46"/>
+      <c r="D31" s="21">
         <f>D11</f>
         <v>3.3</v>
       </c>
-      <c r="E32" s="42">
-        <f>2*IF(OR(D21,D22),E11,0)</f>
+      <c r="E31" s="49">
+        <f>2*IF(OR(D20,D21),E11,0)</f>
         <v>9.6</v>
       </c>
-      <c r="F32" s="42"/>
-      <c r="G32" s="21">
-        <f>D32*E32</f>
+      <c r="F31" s="49"/>
+      <c r="G31" s="21">
+        <f>D31*E31</f>
         <v>31.679999999999996</v>
       </c>
-      <c r="H32" s="21">
-        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)</f>
+      <c r="H31" s="21">
+        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)</f>
         <v>24</v>
       </c>
-      <c r="I32" s="42">
-        <f>G32*H32</f>
+      <c r="I31" s="49">
+        <f>G31*H31</f>
         <v>760.31999999999994</v>
       </c>
-      <c r="J32" s="42"/>
-      <c r="K32" s="42"/>
-      <c r="L32" s="27">
-        <f t="shared" ref="L32:L39" si="1">I32/1000/$D$41</f>
+      <c r="J31" s="49"/>
+      <c r="K31" s="49"/>
+      <c r="L31" s="27">
+        <f t="shared" ref="L31:L38" si="1">I31/1000/$D$40</f>
         <v>0.12999515572906273</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B33" s="40" t="s">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B32" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="41"/>
-      <c r="D33" s="21">
+      <c r="C32" s="46"/>
+      <c r="D32" s="21">
         <f>D12</f>
         <v>3.3</v>
       </c>
-      <c r="E33" s="42">
-        <f>2*IF(OR(D21,D22,D23),E12,0)</f>
+      <c r="E32" s="49">
+        <f>2*IF(OR(D20,D21,D22),E12,0)</f>
         <v>0.8</v>
       </c>
-      <c r="F33" s="42"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="21">
+        <f t="shared" ref="G32:G37" si="2">D32*E32</f>
+        <v>2.64</v>
+      </c>
+      <c r="H32" s="21">
+        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)</f>
+        <v>24</v>
+      </c>
+      <c r="I32" s="49">
+        <f t="shared" ref="I32:I37" si="3">G32*H32</f>
+        <v>63.36</v>
+      </c>
+      <c r="J32" s="49"/>
+      <c r="K32" s="49"/>
+      <c r="L32" s="27">
+        <f t="shared" si="1"/>
+        <v>1.0832929644088564E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B33" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" s="46"/>
+      <c r="D33" s="21">
+        <f>D13</f>
+        <v>5</v>
+      </c>
+      <c r="E33" s="58">
+        <f>IF(OR(D20,D21,D22),E13+(E31+E32)*(D33-D32)/D33,0)</f>
+        <v>9.0360000000000014</v>
+      </c>
+      <c r="F33" s="58"/>
       <c r="G33" s="21">
-        <f t="shared" ref="G33:G38" si="2">D33*E33</f>
-        <v>2.64</v>
+        <f t="shared" si="2"/>
+        <v>45.180000000000007</v>
       </c>
       <c r="H33" s="21">
-        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)</f>
+        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)</f>
         <v>24</v>
       </c>
-      <c r="I33" s="42">
-        <f t="shared" ref="I33:I38" si="3">G33*H33</f>
-        <v>63.36</v>
-      </c>
-      <c r="J33" s="42"/>
-      <c r="K33" s="42"/>
+      <c r="I33" s="49">
+        <f t="shared" si="3"/>
+        <v>1084.3200000000002</v>
+      </c>
+      <c r="J33" s="49"/>
+      <c r="K33" s="49"/>
       <c r="L33" s="27">
         <f t="shared" si="1"/>
-        <v>1.0832929644088564E-2</v>
+        <v>0.18539081868178839</v>
       </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B34" s="40" t="s">
-        <v>26</v>
-      </c>
-      <c r="C34" s="41"/>
+      <c r="B34" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="C34" s="46"/>
       <c r="D34" s="21">
-        <f>D13</f>
+        <f t="shared" ref="D34:E37" si="4">D7</f>
         <v>5</v>
       </c>
-      <c r="E34" s="53">
-        <f>IF(OR(D21,D22,D23),E13+(E32+E33)*(D34-D33)/D34,0)</f>
-        <v>9.0360000000000014</v>
-      </c>
-      <c r="F34" s="53"/>
+      <c r="E34" s="49">
+        <f t="shared" si="4"/>
+        <v>13</v>
+      </c>
+      <c r="F34" s="49"/>
       <c r="G34" s="21">
         <f t="shared" si="2"/>
-        <v>45.180000000000007</v>
+        <v>65</v>
       </c>
       <c r="H34" s="21">
-        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)</f>
         <v>24</v>
       </c>
-      <c r="I34" s="42">
+      <c r="I34" s="49">
         <f t="shared" si="3"/>
-        <v>1084.3200000000002</v>
-      </c>
-      <c r="J34" s="42"/>
-      <c r="K34" s="42"/>
+        <v>1560</v>
+      </c>
+      <c r="J34" s="49"/>
+      <c r="K34" s="49"/>
       <c r="L34" s="27">
         <f t="shared" si="1"/>
-        <v>0.18539081868178839</v>
+        <v>0.26671985866127146</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B35" s="40" t="s">
-        <v>1</v>
-      </c>
-      <c r="C35" s="41"/>
+      <c r="B35" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="C35" s="46"/>
       <c r="D35" s="21">
-        <f t="shared" ref="D35:E38" si="4">D7</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E35" s="42">
+      <c r="E35" s="49">
         <f t="shared" si="4"/>
-        <v>13</v>
-      </c>
-      <c r="F35" s="42"/>
+        <v>16</v>
+      </c>
+      <c r="F35" s="49"/>
       <c r="G35" s="21">
         <f t="shared" si="2"/>
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="H35" s="21">
-        <v>24</v>
-      </c>
-      <c r="I35" s="42">
+        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)-H36-H37</f>
+        <v>22.333333333333336</v>
+      </c>
+      <c r="I35" s="49">
         <f t="shared" si="3"/>
-        <v>1560</v>
-      </c>
-      <c r="J35" s="42"/>
-      <c r="K35" s="42"/>
+        <v>1786.666666666667</v>
+      </c>
+      <c r="J35" s="49"/>
+      <c r="K35" s="49"/>
       <c r="L35" s="27">
         <f t="shared" si="1"/>
-        <v>0.26671985866127146</v>
+        <v>0.30547402615906311</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B36" s="40" t="s">
-        <v>2</v>
-      </c>
-      <c r="C36" s="41"/>
+      <c r="B36" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="C36" s="46"/>
       <c r="D36" s="21">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E36" s="42">
+      <c r="E36" s="49">
         <f t="shared" si="4"/>
-        <v>16</v>
-      </c>
-      <c r="F36" s="42"/>
+        <v>77.5</v>
+      </c>
+      <c r="F36" s="49"/>
       <c r="G36" s="21">
         <f t="shared" si="2"/>
-        <v>80</v>
+        <v>387.5</v>
       </c>
       <c r="H36" s="21">
-        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)-H37-H38</f>
-        <v>22.333333333333336</v>
-      </c>
-      <c r="I36" s="42">
+        <f>IF(NOT(OR(D20,D21)),IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)-H37,IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)*M20*(M21-M22)/3600)</f>
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="I36" s="49">
         <f t="shared" si="3"/>
-        <v>1786.666666666667</v>
-      </c>
-      <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
+        <v>516.66666666666663</v>
+      </c>
+      <c r="J36" s="49"/>
+      <c r="K36" s="49"/>
       <c r="L36" s="27">
         <f t="shared" si="1"/>
-        <v>0.30547402615906311</v>
+        <v>8.8336705325848433E-2</v>
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B37" s="40" t="s">
-        <v>3</v>
-      </c>
-      <c r="C37" s="41"/>
+      <c r="B37" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="46"/>
       <c r="D37" s="21">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E37" s="42">
+      <c r="E37" s="49">
         <f t="shared" si="4"/>
-        <v>77.5</v>
-      </c>
-      <c r="F37" s="42"/>
+        <v>46.5</v>
+      </c>
+      <c r="F37" s="49"/>
       <c r="G37" s="21">
         <f t="shared" si="2"/>
-        <v>387.5</v>
+        <v>232.5</v>
       </c>
       <c r="H37" s="21">
-        <f>IF(NOT(OR(D21,D22)),IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)-H38,IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)*M21*(M22-M23)/3600)</f>
-        <v>1.3333333333333333</v>
-      </c>
-      <c r="I37" s="42">
+        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)*M20*M22/3600</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="I37" s="49">
         <f t="shared" si="3"/>
-        <v>516.66666666666663</v>
-      </c>
-      <c r="J37" s="42"/>
-      <c r="K37" s="42"/>
+        <v>77.5</v>
+      </c>
+      <c r="J37" s="49"/>
+      <c r="K37" s="49"/>
       <c r="L37" s="27">
         <f t="shared" si="1"/>
-        <v>8.8336705325848433E-2</v>
+        <v>1.3250505798877267E-2</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B38" s="40" t="s">
-        <v>4</v>
-      </c>
-      <c r="C38" s="41"/>
+      <c r="B38" s="45" t="s">
+        <v>42</v>
+      </c>
+      <c r="C38" s="46"/>
       <c r="D38" s="21">
-        <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="E38" s="42">
-        <f t="shared" si="4"/>
-        <v>46.5</v>
-      </c>
-      <c r="F38" s="42"/>
-      <c r="G38" s="21">
-        <f t="shared" si="2"/>
-        <v>232.5</v>
+        <f>H21</f>
+        <v>12</v>
+      </c>
+      <c r="E38" s="49">
+        <v>0</v>
+      </c>
+      <c r="F38" s="49"/>
+      <c r="G38" s="32">
+        <f>D38*E38+(1-IF(D38=12,M8,M7))*(SUM(G31:G34)+MAX(G35:G37))</f>
+        <v>111.71999999999998</v>
       </c>
       <c r="H38" s="21">
-        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)*M21*M23/3600</f>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="I38" s="42">
-        <f t="shared" si="3"/>
-        <v>77.5</v>
-      </c>
-      <c r="J38" s="42"/>
-      <c r="K38" s="42"/>
+        <v>24</v>
+      </c>
+      <c r="I38" s="59">
+        <f>D38*E38*H38+(1-IF(D38=12,M8,M7))*SUM(I31:K37)</f>
+        <v>1228.2549999999999</v>
+      </c>
+      <c r="J38" s="59"/>
+      <c r="K38" s="59"/>
       <c r="L38" s="27">
         <f t="shared" si="1"/>
-        <v>1.3250505798877267E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B39" s="40" t="s">
-        <v>42</v>
-      </c>
-      <c r="C39" s="41"/>
-      <c r="D39" s="21">
-        <f>H22</f>
-        <v>12</v>
-      </c>
-      <c r="E39" s="42">
-        <f>IF(D39=12,0,E14)</f>
-        <v>0</v>
-      </c>
-      <c r="F39" s="42"/>
-      <c r="G39" s="32">
-        <f>D39*E39+(1-IF(D39=12,M8,M7))*(SUM(G32:G35)+MAX(G36:G38))</f>
-        <v>111.71999999999998</v>
-      </c>
-      <c r="H39" s="21">
-        <v>24</v>
-      </c>
-      <c r="I39" s="46">
-        <f>D39*E39*H39+(1-IF(D39=12,M8,M7))*SUM(I32:K38)</f>
-        <v>1228.2549999999999</v>
-      </c>
-      <c r="J39" s="46"/>
-      <c r="K39" s="46"/>
-      <c r="L39" s="27">
-        <f t="shared" si="1"/>
         <v>0.20999999999999994</v>
       </c>
     </row>
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B40" s="56" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" s="57"/>
+      <c r="D40" s="3">
+        <f>SUM(I31:I37)/1000</f>
+        <v>5.8488333333333342</v>
+      </c>
+    </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B41" s="51" t="s">
-        <v>30</v>
-      </c>
-      <c r="C41" s="52"/>
-      <c r="D41" s="3">
-        <f>SUM(I32:I38)/1000</f>
-        <v>5.8488333333333342</v>
-      </c>
-    </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B42" s="49" t="s">
+      <c r="B41" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="C42" s="50"/>
-      <c r="D42" s="2" t="str">
-        <f>INT(H23/D41) &amp; "d " &amp; INT(24*MOD(H23,D41)/D41) &amp; "h " &amp; INT(MOD(24*60*MOD(H23,D41)/D41,60)) &amp; "m " &amp; INT(MOD(24*60*60*MOD(H23,D41)/D41,60)) &amp; "s"</f>
+      <c r="C41" s="55"/>
+      <c r="D41" s="2" t="str">
+        <f>INT(H22/D40) &amp; "d " &amp; INT(24*MOD(H22,D40)/D40) &amp; "h " &amp; INT(MOD(24*60*MOD(H22,D40)/D40,60)) &amp; "m " &amp; INT(MOD(24*60*60*MOD(H22,D40)/D40,60)) &amp; "s"</f>
         <v>11d 1h 53m 57s</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="51">
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="K19:N19"/>
-    <mergeCell ref="B2:O2"/>
+  <mergeCells count="49">
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E8:F8"/>
     <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B40:C40"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="I32:K32"/>
-    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="K18:N18"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="B18:D18"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
@@ -2759,47 +2774,12 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E10:F10"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D21:D24">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D20:D23">
       <formula1>"VRAI,FAUX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H22">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H21">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
           <x12ac:list>"3,6",12</x12ac:list>
@@ -2809,7 +2789,7 @@
         </mc:Fallback>
       </mc:AlternateContent>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H21">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H20">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
           <x12ac:list>"20,8","5,4","10,8"</x12ac:list>

</xml_diff>

<commit_message>
Update consumption of RFID reader in search mode & autonomy
</commit_message>
<xml_diff>
--- a/docs/assets/images/User_description/Consumption_and_autonomy.xlsx
+++ b/docs/assets/images/User_description/Consumption_and_autonomy.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\btenaud\Documents\02 - Projet Antenne-Terrier\05 - Documents\2023.04.26 - Estimation conso &amp; autonomie\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\btenaud\Documents\02 - Projet Antenne-Terrier\02 - Git\rfid_m0.wiki\docs\assets\images\User_description\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -74,7 +74,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Current = leakage current of component + Equivalent dissipated current
 Equivalent dissipated current = Power dissipated by regulator / Input voltage 
@@ -279,7 +279,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -361,12 +361,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -655,6 +649,51 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -679,62 +718,17 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -950,28 +944,28 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0.12999515572906273</c:v>
+                  <c:v>0.12816902199870758</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0832929644088564E-2</c:v>
+                  <c:v>1.0680751833225633E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.18539081868178839</c:v>
+                  <c:v>0.18278650296406598</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.26671985866127146</c:v>
+                  <c:v>0.26297305649987357</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.30547402615906311</c:v>
+                  <c:v>0.30118281684600906</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.8336705325848433E-2</c:v>
+                  <c:v>0.10114348326918213</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.3250505798877267E-2</c:v>
+                  <c:v>1.3064366588936026E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.20999999999999994</c:v>
+                  <c:v>0.20999999999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2010,22 +2004,22 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:15" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="44"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="59"/>
     </row>
     <row r="4" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="8" t="s">
@@ -2048,24 +2042,24 @@
       <c r="O4" s="1"/>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="38"/>
+      <c r="C6" s="53"/>
       <c r="D6" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="63" t="s">
+      <c r="E6" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="63"/>
+      <c r="F6" s="37"/>
       <c r="G6" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="37" t="s">
+      <c r="J6" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="K6" s="38"/>
+      <c r="K6" s="53"/>
       <c r="L6" s="30" t="s">
         <v>46</v>
       </c>
@@ -2077,17 +2071,17 @@
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="51"/>
+      <c r="C7" s="63"/>
       <c r="D7" s="17">
         <v>5</v>
       </c>
-      <c r="E7" s="61">
+      <c r="E7" s="41">
         <v>13</v>
       </c>
-      <c r="F7" s="61"/>
+      <c r="F7" s="41"/>
       <c r="G7" s="10">
         <f t="shared" ref="G7:G13" si="0">E7*D7</f>
         <v>65</v>
@@ -2107,17 +2101,17 @@
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="50" t="s">
+      <c r="B8" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="51"/>
+      <c r="C8" s="63"/>
       <c r="D8" s="17">
         <v>5</v>
       </c>
-      <c r="E8" s="61">
+      <c r="E8" s="41">
         <v>16</v>
       </c>
-      <c r="F8" s="61"/>
+      <c r="F8" s="41"/>
       <c r="G8" s="10">
         <f t="shared" si="0"/>
         <v>80</v>
@@ -2137,85 +2131,85 @@
       </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="53"/>
+      <c r="C9" s="45"/>
       <c r="D9" s="17">
         <v>5</v>
       </c>
-      <c r="E9" s="61">
-        <v>77.5</v>
-      </c>
-      <c r="F9" s="61"/>
+      <c r="E9" s="41">
+        <v>90</v>
+      </c>
+      <c r="F9" s="41"/>
       <c r="G9" s="10">
         <f t="shared" si="0"/>
-        <v>387.5</v>
+        <v>450</v>
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="50" t="s">
+      <c r="B10" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="51"/>
+      <c r="C10" s="63"/>
       <c r="D10" s="17">
         <v>5</v>
       </c>
-      <c r="E10" s="61">
+      <c r="E10" s="41">
         <v>46.5</v>
       </c>
-      <c r="F10" s="61"/>
+      <c r="F10" s="41"/>
       <c r="G10" s="10">
         <f t="shared" si="0"/>
         <v>232.5</v>
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="52" t="s">
+      <c r="B11" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="53"/>
+      <c r="C11" s="45"/>
       <c r="D11" s="17">
         <v>3.3</v>
       </c>
-      <c r="E11" s="61">
+      <c r="E11" s="41">
         <v>4.8</v>
       </c>
-      <c r="F11" s="61"/>
+      <c r="F11" s="41"/>
       <c r="G11" s="10">
         <f t="shared" si="0"/>
         <v>15.839999999999998</v>
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="52" t="s">
+      <c r="B12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="53"/>
+      <c r="C12" s="45"/>
       <c r="D12" s="17">
         <v>3.3</v>
       </c>
-      <c r="E12" s="60">
+      <c r="E12" s="43">
         <v>0.4</v>
       </c>
-      <c r="F12" s="60"/>
+      <c r="F12" s="43"/>
       <c r="G12" s="10">
         <f t="shared" si="0"/>
         <v>1.32</v>
       </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="52" t="s">
+      <c r="B13" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="53"/>
+      <c r="C13" s="45"/>
       <c r="D13" s="17">
         <v>5</v>
       </c>
-      <c r="E13" s="60">
+      <c r="E13" s="43">
         <v>5.5</v>
       </c>
-      <c r="F13" s="60"/>
+      <c r="F13" s="43"/>
       <c r="G13" s="10">
         <f t="shared" si="0"/>
         <v>27.5</v>
@@ -2248,25 +2242,25 @@
       <c r="O16" s="1"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="39" t="s">
+      <c r="B18" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="40"/>
-      <c r="D18" s="41"/>
-      <c r="F18" s="39" t="s">
+      <c r="C18" s="55"/>
+      <c r="D18" s="56"/>
+      <c r="F18" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="41"/>
-      <c r="K18" s="39" t="s">
+      <c r="G18" s="55"/>
+      <c r="H18" s="55"/>
+      <c r="I18" s="56"/>
+      <c r="K18" s="54" t="s">
         <v>33</v>
       </c>
-      <c r="L18" s="40" t="s">
+      <c r="L18" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="M18" s="40"/>
-      <c r="N18" s="41"/>
+      <c r="M18" s="55"/>
+      <c r="N18" s="56"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B19" s="11"/>
@@ -2416,17 +2410,17 @@
       <c r="O28" s="1"/>
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B30" s="47" t="s">
+      <c r="B30" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="C30" s="48"/>
+      <c r="C30" s="61"/>
       <c r="D30" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="62" t="s">
+      <c r="E30" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="62"/>
+      <c r="F30" s="42"/>
       <c r="G30" s="25" t="s">
         <v>27</v>
       </c>
@@ -2443,19 +2437,19 @@
       </c>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B31" s="45" t="s">
+      <c r="B31" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C31" s="46"/>
+      <c r="C31" s="39"/>
       <c r="D31" s="21">
         <f>D11</f>
         <v>3.3</v>
       </c>
-      <c r="E31" s="49">
+      <c r="E31" s="40">
         <f>2*IF(OR(D20,D21),E11,0)</f>
         <v>9.6</v>
       </c>
-      <c r="F31" s="49"/>
+      <c r="F31" s="40"/>
       <c r="G31" s="21">
         <f>D31*E31</f>
         <v>31.679999999999996</v>
@@ -2464,31 +2458,31 @@
         <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)</f>
         <v>24</v>
       </c>
-      <c r="I31" s="49">
+      <c r="I31" s="40">
         <f>G31*H31</f>
         <v>760.31999999999994</v>
       </c>
-      <c r="J31" s="49"/>
-      <c r="K31" s="49"/>
+      <c r="J31" s="40"/>
+      <c r="K31" s="40"/>
       <c r="L31" s="27">
         <f t="shared" ref="L31:L38" si="1">I31/1000/$D$40</f>
-        <v>0.12999515572906273</v>
+        <v>0.12816902199870758</v>
       </c>
     </row>
     <row r="32" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B32" s="45" t="s">
+      <c r="B32" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="C32" s="46"/>
+      <c r="C32" s="39"/>
       <c r="D32" s="21">
         <f>D12</f>
         <v>3.3</v>
       </c>
-      <c r="E32" s="49">
+      <c r="E32" s="40">
         <f>2*IF(OR(D20,D21,D22),E12,0)</f>
         <v>0.8</v>
       </c>
-      <c r="F32" s="49"/>
+      <c r="F32" s="40"/>
       <c r="G32" s="21">
         <f t="shared" ref="G32:G37" si="2">D32*E32</f>
         <v>2.64</v>
@@ -2497,31 +2491,31 @@
         <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)</f>
         <v>24</v>
       </c>
-      <c r="I32" s="49">
+      <c r="I32" s="40">
         <f t="shared" ref="I32:I37" si="3">G32*H32</f>
         <v>63.36</v>
       </c>
-      <c r="J32" s="49"/>
-      <c r="K32" s="49"/>
+      <c r="J32" s="40"/>
+      <c r="K32" s="40"/>
       <c r="L32" s="27">
         <f t="shared" si="1"/>
-        <v>1.0832929644088564E-2</v>
+        <v>1.0680751833225633E-2</v>
       </c>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B33" s="45" t="s">
+      <c r="B33" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="46"/>
+      <c r="C33" s="39"/>
       <c r="D33" s="21">
         <f>D13</f>
         <v>5</v>
       </c>
-      <c r="E33" s="58">
+      <c r="E33" s="50">
         <f>IF(OR(D20,D21,D22),E13+(E31+E32)*(D33-D32)/D33,0)</f>
         <v>9.0360000000000014</v>
       </c>
-      <c r="F33" s="58"/>
+      <c r="F33" s="50"/>
       <c r="G33" s="21">
         <f t="shared" si="2"/>
         <v>45.180000000000007</v>
@@ -2530,31 +2524,31 @@
         <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)</f>
         <v>24</v>
       </c>
-      <c r="I33" s="49">
+      <c r="I33" s="40">
         <f t="shared" si="3"/>
         <v>1084.3200000000002</v>
       </c>
-      <c r="J33" s="49"/>
-      <c r="K33" s="49"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="40"/>
       <c r="L33" s="27">
         <f t="shared" si="1"/>
-        <v>0.18539081868178839</v>
+        <v>0.18278650296406598</v>
       </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B34" s="45" t="s">
+      <c r="B34" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="C34" s="46"/>
+      <c r="C34" s="39"/>
       <c r="D34" s="21">
         <f t="shared" ref="D34:E37" si="4">D7</f>
         <v>5</v>
       </c>
-      <c r="E34" s="49">
+      <c r="E34" s="40">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="F34" s="49"/>
+      <c r="F34" s="40"/>
       <c r="G34" s="21">
         <f t="shared" si="2"/>
         <v>65</v>
@@ -2562,31 +2556,31 @@
       <c r="H34" s="21">
         <v>24</v>
       </c>
-      <c r="I34" s="49">
+      <c r="I34" s="40">
         <f t="shared" si="3"/>
         <v>1560</v>
       </c>
-      <c r="J34" s="49"/>
-      <c r="K34" s="49"/>
+      <c r="J34" s="40"/>
+      <c r="K34" s="40"/>
       <c r="L34" s="27">
         <f t="shared" si="1"/>
-        <v>0.26671985866127146</v>
+        <v>0.26297305649987357</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="C35" s="46"/>
+      <c r="C35" s="39"/>
       <c r="D35" s="21">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E35" s="49">
+      <c r="E35" s="40">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="F35" s="49"/>
+      <c r="F35" s="40"/>
       <c r="G35" s="21">
         <f t="shared" si="2"/>
         <v>80</v>
@@ -2595,64 +2589,64 @@
         <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)-H36-H37</f>
         <v>22.333333333333336</v>
       </c>
-      <c r="I35" s="49">
+      <c r="I35" s="40">
         <f t="shared" si="3"/>
         <v>1786.666666666667</v>
       </c>
-      <c r="J35" s="49"/>
-      <c r="K35" s="49"/>
+      <c r="J35" s="40"/>
+      <c r="K35" s="40"/>
       <c r="L35" s="27">
         <f t="shared" si="1"/>
-        <v>0.30547402615906311</v>
+        <v>0.30118281684600906</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B36" s="45" t="s">
+      <c r="B36" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="C36" s="46"/>
+      <c r="C36" s="39"/>
       <c r="D36" s="21">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E36" s="49">
+      <c r="E36" s="40">
         <f t="shared" si="4"/>
-        <v>77.5</v>
-      </c>
-      <c r="F36" s="49"/>
+        <v>90</v>
+      </c>
+      <c r="F36" s="40"/>
       <c r="G36" s="21">
         <f t="shared" si="2"/>
-        <v>387.5</v>
+        <v>450</v>
       </c>
       <c r="H36" s="21">
         <f>IF(NOT(OR(D20,D21)),IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)-H37,IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)*M20*(M21-M22)/3600)</f>
         <v>1.3333333333333333</v>
       </c>
-      <c r="I36" s="49">
+      <c r="I36" s="40">
         <f t="shared" si="3"/>
-        <v>516.66666666666663</v>
-      </c>
-      <c r="J36" s="49"/>
-      <c r="K36" s="49"/>
+        <v>600</v>
+      </c>
+      <c r="J36" s="40"/>
+      <c r="K36" s="40"/>
       <c r="L36" s="27">
         <f t="shared" si="1"/>
-        <v>8.8336705325848433E-2</v>
+        <v>0.10114348326918213</v>
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B37" s="45" t="s">
+      <c r="B37" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="C37" s="46"/>
+      <c r="C37" s="39"/>
       <c r="D37" s="21">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E37" s="49">
+      <c r="E37" s="40">
         <f t="shared" si="4"/>
         <v>46.5</v>
       </c>
-      <c r="F37" s="49"/>
+      <c r="F37" s="40"/>
       <c r="G37" s="21">
         <f t="shared" si="2"/>
         <v>232.5</v>
@@ -2661,87 +2655,86 @@
         <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)*M20*M22/3600</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="I37" s="49">
+      <c r="I37" s="40">
         <f t="shared" si="3"/>
         <v>77.5</v>
       </c>
-      <c r="J37" s="49"/>
-      <c r="K37" s="49"/>
+      <c r="J37" s="40"/>
+      <c r="K37" s="40"/>
       <c r="L37" s="27">
         <f t="shared" si="1"/>
-        <v>1.3250505798877267E-2</v>
+        <v>1.3064366588936026E-2</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B38" s="45" t="s">
+      <c r="B38" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="C38" s="46"/>
+      <c r="C38" s="39"/>
       <c r="D38" s="21">
         <f>H21</f>
         <v>12</v>
       </c>
-      <c r="E38" s="49">
+      <c r="E38" s="40">
         <v>0</v>
       </c>
-      <c r="F38" s="49"/>
+      <c r="F38" s="40"/>
       <c r="G38" s="32">
         <f>D38*E38+(1-IF(D38=12,M8,M7))*(SUM(G31:G34)+MAX(G35:G37))</f>
-        <v>111.71999999999998</v>
+        <v>124.84499999999998</v>
       </c>
       <c r="H38" s="21">
         <v>24</v>
       </c>
-      <c r="I38" s="59">
+      <c r="I38" s="51">
         <f>D38*E38*H38+(1-IF(D38=12,M8,M7))*SUM(I31:K37)</f>
-        <v>1228.2549999999999</v>
-      </c>
-      <c r="J38" s="59"/>
-      <c r="K38" s="59"/>
+        <v>1245.7549999999999</v>
+      </c>
+      <c r="J38" s="51"/>
+      <c r="K38" s="51"/>
       <c r="L38" s="27">
         <f t="shared" si="1"/>
-        <v>0.20999999999999994</v>
+        <v>0.20999999999999996</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B40" s="56" t="s">
+      <c r="B40" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="C40" s="57"/>
+      <c r="C40" s="49"/>
       <c r="D40" s="3">
         <f>SUM(I31:I37)/1000</f>
-        <v>5.8488333333333342</v>
+        <v>5.9321666666666673</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B41" s="54" t="s">
+      <c r="B41" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="C41" s="55"/>
+      <c r="C41" s="47"/>
       <c r="D41" s="2" t="str">
         <f>INT(H22/D40) &amp; "d " &amp; INT(24*MOD(H22,D40)/D40) &amp; "h " &amp; INT(MOD(24*60*MOD(H22,D40)/D40,60)) &amp; "m " &amp; INT(MOD(24*60*60*MOD(H22,D40)/D40,60)) &amp; "s"</f>
-        <v>11d 1h 53m 57s</v>
+        <v>10d 22h 9m 50s</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="K18:N18"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="E32:F32"/>
@@ -2758,22 +2751,23 @@
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="E33:F33"/>
     <mergeCell ref="I38:K38"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="K18:N18"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="E10:F10"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D20:D23">

</xml_diff>

<commit_message>
Update calculation sheet to be more user-friendly
</commit_message>
<xml_diff>
--- a/docs/assets/images/User_description/Consumption_and_autonomy.xlsx
+++ b/docs/assets/images/User_description/Consumption_and_autonomy.xlsx
@@ -38,7 +38,7 @@
     <author>benjamin tenaud</author>
   </authors>
   <commentList>
-    <comment ref="M7" authorId="0" shapeId="0">
+    <comment ref="M8" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -53,7 +53,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M8" authorId="0" shapeId="0">
+    <comment ref="M9" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -67,7 +67,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E33" authorId="0" shapeId="0">
+    <comment ref="E34" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -83,7 +83,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G38" authorId="0" shapeId="0">
+    <comment ref="G39" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -97,7 +97,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I38" authorId="0" shapeId="0">
+    <comment ref="I39" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -116,7 +116,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="50">
   <si>
     <t>Component</t>
   </si>
@@ -274,12 +274,18 @@
   <si>
     <t>Duration [h]</t>
   </si>
+  <si>
+    <t>configurable inputs according to your configuration</t>
+  </si>
+  <si>
+    <t>Datasheet password : Mibe2023</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -362,8 +368,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -403,6 +417,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -573,7 +593,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -585,9 +605,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -595,15 +612,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -640,95 +651,121 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -907,7 +944,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Feuil1!$B$31:$C$38</c:f>
+              <c:f>Feuil1!$B$32:$C$39</c:f>
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
@@ -939,7 +976,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Feuil1!$L$31:$L$38</c:f>
+              <c:f>Feuil1!$L$32:$L$39</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="8"/>
@@ -965,7 +1002,7 @@
                   <c:v>1.3064366588936026E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.20999999999999996</c:v>
+                  <c:v>7.9999999999999946E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1691,13 +1728,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>390525</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>104774</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>266700</xdr:colOff>
-      <xdr:row>59</xdr:row>
+      <xdr:row>60</xdr:row>
       <xdr:rowOff>152399</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1983,7 +2020,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:O41"/>
+  <dimension ref="B1:O42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2004,776 +2041,802 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:15" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="59"/>
-    </row>
-    <row r="4" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B4" s="8" t="s">
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="38"/>
+    </row>
+    <row r="3" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="66" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="65"/>
+      <c r="L3" s="65"/>
+      <c r="M3" s="65"/>
+      <c r="N3" s="65"/>
+      <c r="O3" s="65"/>
+    </row>
+    <row r="5" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="8" t="s">
+      <c r="C5" s="15"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="52" t="s">
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B7" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="53"/>
-      <c r="D6" s="22" t="s">
+      <c r="C7" s="32"/>
+      <c r="D7" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="E7" s="55" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="37"/>
-      <c r="G6" s="23" t="s">
+      <c r="F7" s="55"/>
+      <c r="G7" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="52" t="s">
+      <c r="J7" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="K6" s="53"/>
-      <c r="L6" s="30" t="s">
+      <c r="K7" s="32"/>
+      <c r="L7" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="M6" s="33" t="s">
+      <c r="M7" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="N6" s="31" t="s">
+      <c r="N7" s="28" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="62" t="s">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B8" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="63"/>
-      <c r="D7" s="17">
+      <c r="C8" s="45"/>
+      <c r="D8" s="60">
         <v>5</v>
       </c>
-      <c r="E7" s="41">
+      <c r="E8" s="61">
         <v>13</v>
       </c>
-      <c r="F7" s="41"/>
-      <c r="G7" s="10">
-        <f t="shared" ref="G7:G13" si="0">E7*D7</f>
+      <c r="F8" s="61"/>
+      <c r="G8" s="9">
+        <f t="shared" ref="G8:G14" si="0">E8*D8</f>
         <v>65</v>
       </c>
-      <c r="J7" s="9" t="s">
+      <c r="J8" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="28"/>
-      <c r="L7" s="28" t="s">
+      <c r="K8" s="25"/>
+      <c r="L8" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="M7" s="34">
+      <c r="M8" s="63">
         <v>0.92</v>
       </c>
-      <c r="N7" s="29" t="s">
+      <c r="N8" s="26" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="62" t="s">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B9" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="63"/>
-      <c r="D8" s="17">
+      <c r="C9" s="45"/>
+      <c r="D9" s="60">
         <v>5</v>
       </c>
-      <c r="E8" s="41">
+      <c r="E9" s="61">
         <v>16</v>
       </c>
-      <c r="F8" s="41"/>
-      <c r="G8" s="10">
+      <c r="F9" s="61"/>
+      <c r="G9" s="9">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J9" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1" t="s">
+      <c r="K9" s="1"/>
+      <c r="L9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="M8" s="35">
+      <c r="M9" s="64">
         <v>0.79</v>
       </c>
-      <c r="N8" s="16" t="s">
+      <c r="N9" s="14" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="44" t="s">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B10" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="45"/>
-      <c r="D9" s="17">
+      <c r="C10" s="47"/>
+      <c r="D10" s="60">
         <v>5</v>
       </c>
-      <c r="E9" s="41">
+      <c r="E10" s="61">
         <v>90</v>
       </c>
-      <c r="F9" s="41"/>
-      <c r="G9" s="10">
+      <c r="F10" s="61"/>
+      <c r="G10" s="9">
         <f t="shared" si="0"/>
         <v>450</v>
       </c>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="62" t="s">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B11" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="63"/>
-      <c r="D10" s="17">
+      <c r="C11" s="45"/>
+      <c r="D11" s="60">
         <v>5</v>
       </c>
-      <c r="E10" s="41">
+      <c r="E11" s="61">
         <v>46.5</v>
       </c>
-      <c r="F10" s="41"/>
-      <c r="G10" s="10">
+      <c r="F11" s="61"/>
+      <c r="G11" s="9">
         <f t="shared" si="0"/>
         <v>232.5</v>
       </c>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="44" t="s">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B12" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="45"/>
-      <c r="D11" s="17">
+      <c r="C12" s="47"/>
+      <c r="D12" s="60">
         <v>3.3</v>
       </c>
-      <c r="E11" s="41">
+      <c r="E12" s="61">
         <v>4.8</v>
       </c>
-      <c r="F11" s="41"/>
-      <c r="G11" s="10">
+      <c r="F12" s="61"/>
+      <c r="G12" s="9">
         <f t="shared" si="0"/>
         <v>15.839999999999998</v>
       </c>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="44" t="s">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B13" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="45"/>
-      <c r="D12" s="17">
+      <c r="C13" s="47"/>
+      <c r="D13" s="60">
         <v>3.3</v>
       </c>
-      <c r="E12" s="43">
+      <c r="E13" s="62">
         <v>0.4</v>
       </c>
-      <c r="F12" s="43"/>
-      <c r="G12" s="10">
+      <c r="F13" s="62"/>
+      <c r="G13" s="9">
         <f t="shared" si="0"/>
         <v>1.32</v>
       </c>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="44" t="s">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B14" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="45"/>
-      <c r="D13" s="17">
+      <c r="C14" s="47"/>
+      <c r="D14" s="60">
         <v>5</v>
       </c>
-      <c r="E13" s="43">
+      <c r="E14" s="62">
         <v>5.5</v>
       </c>
-      <c r="F13" s="43"/>
-      <c r="G13" s="10">
+      <c r="F14" s="62"/>
+      <c r="G14" s="9">
         <f t="shared" si="0"/>
         <v>27.5</v>
       </c>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="4" t="s">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B15" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="4"/>
-    </row>
-    <row r="16" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B16" s="8" t="s">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B16" s="4"/>
+    </row>
+    <row r="17" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="54" t="s">
+      <c r="C17" s="15"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B19" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="55"/>
-      <c r="D18" s="56"/>
-      <c r="F18" s="54" t="s">
+      <c r="C19" s="34"/>
+      <c r="D19" s="35"/>
+      <c r="F19" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="G18" s="55"/>
-      <c r="H18" s="55"/>
-      <c r="I18" s="56"/>
-      <c r="K18" s="54" t="s">
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="35"/>
+      <c r="K19" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="L18" s="55" t="s">
+      <c r="L19" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="M18" s="55"/>
-      <c r="N18" s="56"/>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="11"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="15"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="20"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="20"/>
+      <c r="M19" s="34"/>
+      <c r="N19" s="35"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B20" s="12"/>
-      <c r="C20" s="5" t="s">
+      <c r="B20" s="10"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="13"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="17"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="17"/>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B21" s="11"/>
+      <c r="C21" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="13" t="b">
+      <c r="D21" s="57" t="b">
         <v>1</v>
       </c>
-      <c r="F20" s="12"/>
-      <c r="G20" s="5" t="s">
+      <c r="F21" s="11"/>
+      <c r="G21" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H20" s="7">
-        <v>5.4</v>
-      </c>
-      <c r="I20" s="20"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="5" t="s">
+      <c r="H21" s="58">
+        <v>20.8</v>
+      </c>
+      <c r="I21" s="17"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="M20" s="7">
+      <c r="M21" s="58">
         <v>50</v>
       </c>
-      <c r="N20" s="20"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B21" s="12"/>
-      <c r="C21" s="5" t="s">
+      <c r="N21" s="17"/>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B22" s="11"/>
+      <c r="C22" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="13" t="b">
+      <c r="D22" s="57" t="b">
         <v>1</v>
       </c>
-      <c r="F21" s="12"/>
-      <c r="G21" s="5" t="s">
+      <c r="F22" s="11"/>
+      <c r="G22" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H21" s="7">
-        <v>12</v>
-      </c>
-      <c r="I21" s="20"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="5" t="s">
+      <c r="H22" s="58">
+        <v>3.6</v>
+      </c>
+      <c r="I22" s="17"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="M21" s="7">
+      <c r="M22" s="58">
         <v>5</v>
       </c>
-      <c r="N21" s="20"/>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B22" s="12"/>
-      <c r="C22" s="5" t="s">
+      <c r="N22" s="17"/>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B23" s="11"/>
+      <c r="C23" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D22" s="13" t="b">
+      <c r="D23" s="57" t="b">
         <v>0</v>
       </c>
-      <c r="F22" s="12"/>
-      <c r="G22" s="5" t="s">
+      <c r="F23" s="11"/>
+      <c r="G23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="19">
-        <f>H20*H21</f>
-        <v>64.800000000000011</v>
-      </c>
-      <c r="I22" s="20"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="5" t="s">
+      <c r="H23" s="16">
+        <f>H21*H22</f>
+        <v>74.88000000000001</v>
+      </c>
+      <c r="I23" s="17"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="M22" s="36">
+      <c r="M23" s="59">
         <v>1</v>
       </c>
-      <c r="N22" s="20"/>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="12"/>
-      <c r="C23" s="5" t="s">
+      <c r="N23" s="17"/>
+    </row>
+    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B24" s="11"/>
+      <c r="C24" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="13" t="b">
+      <c r="D24" s="57" t="b">
         <v>0</v>
       </c>
-      <c r="F23" s="14"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="16"/>
-      <c r="K23" s="14"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="16"/>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="12"/>
-      <c r="C24" s="5" t="s">
+      <c r="F24" s="12"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="14"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="14"/>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B25" s="11"/>
+      <c r="C25" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="13">
+      <c r="D25" s="57">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="12"/>
-      <c r="C25" s="5" t="s">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B26" s="11"/>
+      <c r="C26" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D25" s="13">
+      <c r="D26" s="57">
         <v>20</v>
       </c>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="14"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="16"/>
-    </row>
-    <row r="28" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B28" s="8" t="s">
+      <c r="F26" s="56" t="s">
+        <v>48</v>
+      </c>
+      <c r="G26" s="56"/>
+      <c r="H26" s="56"/>
+      <c r="I26" s="56"/>
+    </row>
+    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B27" s="12"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="14"/>
+    </row>
+    <row r="29" spans="2:15" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B29" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-      <c r="K28" s="1"/>
-      <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
-      <c r="N28" s="1"/>
-      <c r="O28" s="1"/>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B30" s="60" t="s">
+      <c r="C29" s="15"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+    </row>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B31" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="C30" s="61"/>
-      <c r="D30" s="25" t="s">
+      <c r="C31" s="42"/>
+      <c r="D31" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="42" t="s">
+      <c r="E31" s="54" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="42"/>
-      <c r="G30" s="25" t="s">
+      <c r="F31" s="54"/>
+      <c r="G31" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="H30" s="25" t="s">
+      <c r="H31" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="I30" s="24" t="s">
+      <c r="I31" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="J30" s="24"/>
-      <c r="K30" s="24"/>
-      <c r="L30" s="26" t="s">
+      <c r="J31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="23" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B31" s="38" t="s">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B32" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C31" s="39"/>
-      <c r="D31" s="21">
-        <f>D11</f>
-        <v>3.3</v>
-      </c>
-      <c r="E31" s="40">
-        <f>2*IF(OR(D20,D21),E11,0)</f>
-        <v>9.6</v>
-      </c>
-      <c r="F31" s="40"/>
-      <c r="G31" s="21">
-        <f>D31*E31</f>
-        <v>31.679999999999996</v>
-      </c>
-      <c r="H31" s="21">
-        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)</f>
-        <v>24</v>
-      </c>
-      <c r="I31" s="40">
-        <f>G31*H31</f>
-        <v>760.31999999999994</v>
-      </c>
-      <c r="J31" s="40"/>
-      <c r="K31" s="40"/>
-      <c r="L31" s="27">
-        <f t="shared" ref="L31:L38" si="1">I31/1000/$D$40</f>
-        <v>0.12816902199870758</v>
-      </c>
-    </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B32" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" s="39"/>
-      <c r="D32" s="21">
+      <c r="C32" s="40"/>
+      <c r="D32" s="18">
         <f>D12</f>
         <v>3.3</v>
       </c>
-      <c r="E32" s="40">
-        <f>2*IF(OR(D20,D21,D22),E12,0)</f>
+      <c r="E32" s="43">
+        <f>2*IF(OR(D21,D22),E12,0)</f>
+        <v>9.6</v>
+      </c>
+      <c r="F32" s="43"/>
+      <c r="G32" s="18">
+        <f>D32*E32</f>
+        <v>31.679999999999996</v>
+      </c>
+      <c r="H32" s="18">
+        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)</f>
+        <v>24</v>
+      </c>
+      <c r="I32" s="43">
+        <f>G32*H32</f>
+        <v>760.31999999999994</v>
+      </c>
+      <c r="J32" s="43"/>
+      <c r="K32" s="43"/>
+      <c r="L32" s="24">
+        <f t="shared" ref="L32:L39" si="1">I32/1000/$D$41</f>
+        <v>0.12816902199870758</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B33" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="C33" s="40"/>
+      <c r="D33" s="18">
+        <f>D13</f>
+        <v>3.3</v>
+      </c>
+      <c r="E33" s="43">
+        <f>2*IF(OR(D21,D22,D23),E13,0)</f>
         <v>0.8</v>
       </c>
-      <c r="F32" s="40"/>
-      <c r="G32" s="21">
-        <f t="shared" ref="G32:G37" si="2">D32*E32</f>
+      <c r="F33" s="43"/>
+      <c r="G33" s="18">
+        <f t="shared" ref="G33:G38" si="2">D33*E33</f>
         <v>2.64</v>
       </c>
-      <c r="H32" s="21">
-        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)</f>
+      <c r="H33" s="18">
+        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)</f>
         <v>24</v>
       </c>
-      <c r="I32" s="40">
-        <f t="shared" ref="I32:I37" si="3">G32*H32</f>
+      <c r="I33" s="43">
+        <f t="shared" ref="I33:I38" si="3">G33*H33</f>
         <v>63.36</v>
       </c>
-      <c r="J32" s="40"/>
-      <c r="K32" s="40"/>
-      <c r="L32" s="27">
+      <c r="J33" s="43"/>
+      <c r="K33" s="43"/>
+      <c r="L33" s="24">
         <f t="shared" si="1"/>
         <v>1.0680751833225633E-2</v>
       </c>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B33" s="38" t="s">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B34" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="39"/>
-      <c r="D33" s="21">
-        <f>D13</f>
+      <c r="C34" s="40"/>
+      <c r="D34" s="18">
+        <f>D14</f>
         <v>5</v>
       </c>
-      <c r="E33" s="50">
-        <f>IF(OR(D20,D21,D22),E13+(E31+E32)*(D33-D32)/D33,0)</f>
+      <c r="E34" s="52">
+        <f>IF(OR(D21,D22,D23),E14+(E32+E33)*(D34-D33)/D34,0)</f>
         <v>9.0360000000000014</v>
       </c>
-      <c r="F33" s="50"/>
-      <c r="G33" s="21">
+      <c r="F34" s="52"/>
+      <c r="G34" s="18">
         <f t="shared" si="2"/>
         <v>45.180000000000007</v>
       </c>
-      <c r="H33" s="21">
-        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)</f>
+      <c r="H34" s="18">
+        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)</f>
         <v>24</v>
       </c>
-      <c r="I33" s="40">
+      <c r="I34" s="43">
         <f t="shared" si="3"/>
         <v>1084.3200000000002</v>
       </c>
-      <c r="J33" s="40"/>
-      <c r="K33" s="40"/>
-      <c r="L33" s="27">
+      <c r="J34" s="43"/>
+      <c r="K34" s="43"/>
+      <c r="L34" s="24">
         <f t="shared" si="1"/>
         <v>0.18278650296406598</v>
       </c>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B34" s="38" t="s">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B35" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C34" s="39"/>
-      <c r="D34" s="21">
-        <f t="shared" ref="D34:E37" si="4">D7</f>
+      <c r="C35" s="40"/>
+      <c r="D35" s="18">
+        <f t="shared" ref="D35:E38" si="4">D8</f>
         <v>5</v>
       </c>
-      <c r="E34" s="40">
+      <c r="E35" s="43">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="F34" s="40"/>
-      <c r="G34" s="21">
+      <c r="F35" s="43"/>
+      <c r="G35" s="18">
         <f t="shared" si="2"/>
         <v>65</v>
       </c>
-      <c r="H34" s="21">
+      <c r="H35" s="18">
         <v>24</v>
       </c>
-      <c r="I34" s="40">
+      <c r="I35" s="43">
         <f t="shared" si="3"/>
         <v>1560</v>
       </c>
-      <c r="J34" s="40"/>
-      <c r="K34" s="40"/>
-      <c r="L34" s="27">
+      <c r="J35" s="43"/>
+      <c r="K35" s="43"/>
+      <c r="L35" s="24">
         <f t="shared" si="1"/>
         <v>0.26297305649987357</v>
       </c>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B35" s="38" t="s">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B36" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="C35" s="39"/>
-      <c r="D35" s="21">
+      <c r="C36" s="40"/>
+      <c r="D36" s="18">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E35" s="40">
+      <c r="E36" s="43">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="F35" s="40"/>
-      <c r="G35" s="21">
+      <c r="F36" s="43"/>
+      <c r="G36" s="18">
         <f t="shared" si="2"/>
         <v>80</v>
       </c>
-      <c r="H35" s="21">
-        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)-H36-H37</f>
+      <c r="H36" s="18">
+        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)-H37-H38</f>
         <v>22.333333333333336</v>
       </c>
-      <c r="I35" s="40">
+      <c r="I36" s="43">
         <f t="shared" si="3"/>
         <v>1786.666666666667</v>
       </c>
-      <c r="J35" s="40"/>
-      <c r="K35" s="40"/>
-      <c r="L35" s="27">
+      <c r="J36" s="43"/>
+      <c r="K36" s="43"/>
+      <c r="L36" s="24">
         <f t="shared" si="1"/>
         <v>0.30118281684600906</v>
       </c>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B36" s="38" t="s">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B37" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="C36" s="39"/>
-      <c r="D36" s="21">
+      <c r="C37" s="40"/>
+      <c r="D37" s="18">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E36" s="40">
+      <c r="E37" s="43">
         <f t="shared" si="4"/>
         <v>90</v>
       </c>
-      <c r="F36" s="40"/>
-      <c r="G36" s="21">
+      <c r="F37" s="43"/>
+      <c r="G37" s="18">
         <f t="shared" si="2"/>
         <v>450</v>
       </c>
-      <c r="H36" s="21">
-        <f>IF(NOT(OR(D20,D21)),IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)-H37,IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)*M20*(M21-M22)/3600)</f>
+      <c r="H37" s="18">
+        <f>IF(NOT(OR(D21,D22)),IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)-H38,IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)*M21*(M22-M23)/3600)</f>
         <v>1.3333333333333333</v>
       </c>
-      <c r="I36" s="40">
+      <c r="I37" s="43">
         <f t="shared" si="3"/>
         <v>600</v>
       </c>
-      <c r="J36" s="40"/>
-      <c r="K36" s="40"/>
-      <c r="L36" s="27">
+      <c r="J37" s="43"/>
+      <c r="K37" s="43"/>
+      <c r="L37" s="24">
         <f t="shared" si="1"/>
         <v>0.10114348326918213</v>
       </c>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B37" s="38" t="s">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B38" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="C37" s="39"/>
-      <c r="D37" s="21">
+      <c r="C38" s="40"/>
+      <c r="D38" s="18">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="E37" s="40">
+      <c r="E38" s="43">
         <f t="shared" si="4"/>
         <v>46.5</v>
       </c>
-      <c r="F37" s="40"/>
-      <c r="G37" s="21">
+      <c r="F38" s="43"/>
+      <c r="G38" s="18">
         <f t="shared" si="2"/>
         <v>232.5</v>
       </c>
-      <c r="H37" s="21">
-        <f>IF($D$23,IF($D$25&gt;$D$24,$D$25-$D$24,24-$D$24+$D$25),24)*M20*M22/3600</f>
+      <c r="H38" s="18">
+        <f>IF($D$24,IF($D$26&gt;$D$25,$D$26-$D$25,24-$D$25+$D$26),24)*M21*M23/3600</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="I37" s="40">
+      <c r="I38" s="43">
         <f t="shared" si="3"/>
         <v>77.5</v>
       </c>
-      <c r="J37" s="40"/>
-      <c r="K37" s="40"/>
-      <c r="L37" s="27">
+      <c r="J38" s="43"/>
+      <c r="K38" s="43"/>
+      <c r="L38" s="24">
         <f t="shared" si="1"/>
         <v>1.3064366588936026E-2</v>
       </c>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B38" s="38" t="s">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B39" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="C38" s="39"/>
-      <c r="D38" s="21">
-        <f>H21</f>
-        <v>12</v>
-      </c>
-      <c r="E38" s="40">
+      <c r="C39" s="40"/>
+      <c r="D39" s="18">
+        <f>H22</f>
+        <v>3.6</v>
+      </c>
+      <c r="E39" s="43">
         <v>0</v>
       </c>
-      <c r="F38" s="40"/>
-      <c r="G38" s="32">
-        <f>D38*E38+(1-IF(D38=12,M8,M7))*(SUM(G31:G34)+MAX(G35:G37))</f>
-        <v>124.84499999999998</v>
-      </c>
-      <c r="H38" s="21">
+      <c r="F39" s="43"/>
+      <c r="G39" s="29">
+        <f>D39*E39+(1-IF(D39=12,M9,M8))*(SUM(G32:G35)+MAX(G36:G38))</f>
+        <v>47.559999999999974</v>
+      </c>
+      <c r="H39" s="18">
         <v>24</v>
       </c>
-      <c r="I38" s="51">
-        <f>D38*E38*H38+(1-IF(D38=12,M8,M7))*SUM(I31:K37)</f>
-        <v>1245.7549999999999</v>
-      </c>
-      <c r="J38" s="51"/>
-      <c r="K38" s="51"/>
-      <c r="L38" s="27">
+      <c r="I39" s="53">
+        <f>D39*E39*H39+(1-IF(D39=12,M9,M8))*SUM(I32:K38)</f>
+        <v>474.5733333333331</v>
+      </c>
+      <c r="J39" s="53"/>
+      <c r="K39" s="53"/>
+      <c r="L39" s="24">
         <f t="shared" si="1"/>
-        <v>0.20999999999999996</v>
-      </c>
-    </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B40" s="48" t="s">
+        <v>7.9999999999999946E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B41" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="C40" s="49"/>
-      <c r="D40" s="3">
-        <f>SUM(I31:I37)/1000</f>
+      <c r="C41" s="51"/>
+      <c r="D41" s="3">
+        <f>SUM(I32:I38)/1000</f>
         <v>5.9321666666666673</v>
       </c>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B41" s="46" t="s">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B42" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="C41" s="47"/>
-      <c r="D41" s="2" t="str">
-        <f>INT(H22/D40) &amp; "d " &amp; INT(24*MOD(H22,D40)/D40) &amp; "h " &amp; INT(MOD(24*60*MOD(H22,D40)/D40,60)) &amp; "m " &amp; INT(MOD(24*60*60*MOD(H22,D40)/D40,60)) &amp; "s"</f>
-        <v>10d 22h 9m 50s</v>
+      <c r="C42" s="49"/>
+      <c r="D42" s="2" t="str">
+        <f>INT(H23/D41) &amp; "d " &amp; INT(24*MOD(H23,D41)/D41) &amp; "h " &amp; INT(MOD(24*60*MOD(H23,D41)/D41,60)) &amp; "m " &amp; INT(MOD(24*60*60*MOD(H23,D41)/D41,60)) &amp; "s"</f>
+        <v>12d 14h 56m 41s</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="49">
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="K18:N18"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="3r+y+YLvfxQt766h4LylUbJqi+CCqL94Do19g1bDiPJ5BGxFRU7OP4fUrLNp1Yu9s+pza3b1Sw+xcv2P55c30g==" saltValue="UizgRQRSvswNGK2BavuSuw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <mergeCells count="50">
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="I37:K37"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="I36:K36"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="I33:K33"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="I39:K39"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="K19:N19"/>
     <mergeCell ref="B2:O2"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E11:F11"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="E10:F10"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D20:D23">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D21:D24">
       <formula1>"VRAI,FAUX"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H21">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H22">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
           <x12ac:list>"3,6",12</x12ac:list>
@@ -2783,7 +2846,7 @@
         </mc:Fallback>
       </mc:AlternateContent>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H20">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H21">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
           <x12ac:list>"20,8","5,4","10,8"</x12ac:list>

</xml_diff>